<commit_message>
Roosevelt DE: metodologia Barrio Obrero (consolidado Camara Comercio + stock activo + 3 componentes establecimientos/ingresos/empleo); nuevo build_de_roosevelt.py; Excel regenerado (DE 54.2/91.4/95.7/95.7, ITT 51.4/66.5/65.6/79.4)
</commit_message>
<xml_diff>
--- a/outputs/itt_roosevelt/ITT_Roosevelt_Consolidado.xlsx
+++ b/outputs/itt_roosevelt/ITT_Roosevelt_Consolidado.xlsx
@@ -483,10 +483,10 @@
         <v>76.5</v>
       </c>
       <c r="F2" t="n">
-        <v>91.61</v>
+        <v>54.18</v>
       </c>
       <c r="G2" t="n">
-        <v>57.03</v>
+        <v>51.42</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -511,10 +511,10 @@
         <v>89.5</v>
       </c>
       <c r="F3" t="n">
-        <v>95.65000000000001</v>
+        <v>91.34999999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>67.11</v>
+        <v>66.45999999999999</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -539,10 +539,10 @@
         <v>89.5</v>
       </c>
       <c r="F4" t="n">
-        <v>100</v>
+        <v>95.65000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>66.2</v>
+        <v>65.55</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -567,14 +567,14 @@
         <v>88.2</v>
       </c>
       <c r="F5" t="n">
-        <v>100</v>
+        <v>95.65000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>80.08</v>
+        <v>79.43000000000001</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Escala</t>
+          <t>Transformacion</t>
         </is>
       </c>
     </row>
@@ -632,7 +632,7 @@
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>62.26</v>
+        <v>56.64</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -651,7 +651,7 @@
         <v>2</v>
       </c>
       <c r="D3" t="n">
-        <v>62.79</v>
+        <v>57.17</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -670,7 +670,7 @@
         <v>3</v>
       </c>
       <c r="D4" t="n">
-        <v>73.14</v>
+        <v>67.52</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -689,7 +689,7 @@
         <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>60.85</v>
+        <v>55.23</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -708,7 +708,7 @@
         <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>66.76000000000001</v>
+        <v>66.12</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -727,7 +727,7 @@
         <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>70.70999999999999</v>
+        <v>70.06999999999999</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -746,7 +746,7 @@
         <v>3</v>
       </c>
       <c r="D8" t="n">
-        <v>78.31</v>
+        <v>77.67</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -765,7 +765,7 @@
         <v>4</v>
       </c>
       <c r="D9" t="n">
-        <v>83.15000000000001</v>
+        <v>82.51000000000001</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -784,7 +784,7 @@
         <v>1</v>
       </c>
       <c r="D10" t="n">
-        <v>73.97</v>
+        <v>73.31999999999999</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -803,7 +803,7 @@
         <v>2</v>
       </c>
       <c r="D11" t="n">
-        <v>70.95</v>
+        <v>70.3</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -822,7 +822,7 @@
         <v>3</v>
       </c>
       <c r="D12" t="n">
-        <v>71.31999999999999</v>
+        <v>70.67</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -841,7 +841,7 @@
         <v>4</v>
       </c>
       <c r="D13" t="n">
-        <v>73.90000000000001</v>
+        <v>73.25</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -860,7 +860,7 @@
         <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>81.09999999999999</v>
+        <v>80.45</v>
       </c>
       <c r="E14" t="b">
         <v>1</v>
@@ -2189,7 +2189,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Proxy retrospectivo</t>
+          <t>Real (stock activo consolidado)</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -2211,13 +2211,13 @@
         <v>78.09</v>
       </c>
       <c r="I2" t="n">
-        <v>97.09999999999999</v>
+        <v>84.43000000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>99.64</v>
+        <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>91.61</v>
+        <v>54.18</v>
       </c>
     </row>
     <row r="3">
@@ -2226,7 +2226,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Proxy retrospectivo</t>
+          <t>Real (stock activo consolidado)</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -2248,13 +2248,13 @@
         <v>88.23999999999999</v>
       </c>
       <c r="I3" t="n">
-        <v>98.72</v>
+        <v>85.84</v>
       </c>
       <c r="J3" t="n">
-        <v>100</v>
+        <v>99.97</v>
       </c>
       <c r="K3" t="n">
-        <v>95.65000000000001</v>
+        <v>91.34999999999999</v>
       </c>
     </row>
     <row r="4">
@@ -2263,7 +2263,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Real</t>
+          <t>Real (stock activo consolidado)</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -2285,13 +2285,13 @@
         <v>100</v>
       </c>
       <c r="I4" t="n">
-        <v>100</v>
+        <v>86.95999999999999</v>
       </c>
       <c r="J4" t="n">
         <v>100</v>
       </c>
       <c r="K4" t="n">
-        <v>100</v>
+        <v>95.65000000000001</v>
       </c>
     </row>
     <row r="5">
@@ -2300,7 +2300,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Proxy referencial = 2025</t>
+          <t>Real (stock activo consolidado)</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -2322,13 +2322,13 @@
         <v>100</v>
       </c>
       <c r="I5" t="n">
-        <v>100</v>
+        <v>86.95999999999999</v>
       </c>
       <c r="J5" t="n">
         <v>100</v>
       </c>
       <c r="K5" t="n">
-        <v>100</v>
+        <v>95.65000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Roosevelt DE: integracion real data 2026 CCC (CSV 20260929 fechas/cancelaciones hasta sep-2026 + empleo PERSONAL_OCUPADO del xlsx), stock activo trimestral 2026 Q1-Q3, grafica + hoja DesEco_Trim_2026, 2026 marcado Parcial; DE 53.8/91.0/95.7/93.7
</commit_message>
<xml_diff>
--- a/outputs/itt_roosevelt/ITT_Roosevelt_Consolidado.xlsx
+++ b/outputs/itt_roosevelt/ITT_Roosevelt_Consolidado.xlsx
@@ -15,7 +15,8 @@
     <sheet name="Entorno_Urbano" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Educacion" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Desarrollo_Economico" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Indicadores_Trimestrales" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="DesEco_Trim_2026" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Indicadores_Trimestrales" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -483,10 +484,10 @@
         <v>76.5</v>
       </c>
       <c r="F2" t="n">
-        <v>54.18</v>
+        <v>53.75</v>
       </c>
       <c r="G2" t="n">
-        <v>51.42</v>
+        <v>51.35</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -511,10 +512,10 @@
         <v>89.5</v>
       </c>
       <c r="F3" t="n">
-        <v>91.34999999999999</v>
+        <v>91.03</v>
       </c>
       <c r="G3" t="n">
-        <v>66.45999999999999</v>
+        <v>66.41</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -567,16 +568,649 @@
         <v>88.2</v>
       </c>
       <c r="F5" t="n">
-        <v>95.65000000000001</v>
+        <v>93.68000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>79.43000000000001</v>
+        <v>79.13</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>Transformacion</t>
         </is>
       </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>año</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>trimestre</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>homicidios</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>hurtos</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>siniestralidad</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>lesionados</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>mortales</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>vif</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>rinas</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>periodo</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>spa</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>57</v>
+      </c>
+      <c r="E2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F2" t="n">
+        <v>7</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>2023-Q1</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>68</v>
+      </c>
+      <c r="E3" t="n">
+        <v>8</v>
+      </c>
+      <c r="F3" t="n">
+        <v>7</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2023-Q2</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>64</v>
+      </c>
+      <c r="E4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I4" t="n">
+        <v>6</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>2023-Q3</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>56</v>
+      </c>
+      <c r="E5" t="n">
+        <v>9</v>
+      </c>
+      <c r="F5" t="n">
+        <v>8</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I5" t="n">
+        <v>4</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>2023-Q4</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>61</v>
+      </c>
+      <c r="E6" t="n">
+        <v>7</v>
+      </c>
+      <c r="F6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" t="n">
+        <v>5</v>
+      </c>
+      <c r="I6" t="n">
+        <v>4</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2024-Q1</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>76</v>
+      </c>
+      <c r="E7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F7" t="n">
+        <v>5</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>2024-Q2</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>73</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>3</v>
+      </c>
+      <c r="I8" t="n">
+        <v>6</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2024-Q3</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B9" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>64</v>
+      </c>
+      <c r="E9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>2024-Q4</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>48</v>
+      </c>
+      <c r="E10" t="n">
+        <v>9</v>
+      </c>
+      <c r="F10" t="n">
+        <v>9</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" t="n">
+        <v>3</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>2025-Q1</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B11" t="n">
+        <v>2</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>56</v>
+      </c>
+      <c r="E11" t="n">
+        <v>6</v>
+      </c>
+      <c r="F11" t="n">
+        <v>5</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" t="n">
+        <v>2</v>
+      </c>
+      <c r="I11" t="n">
+        <v>2</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>2025-Q2</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B12" t="n">
+        <v>3</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="n">
+        <v>57</v>
+      </c>
+      <c r="E12" t="n">
+        <v>5</v>
+      </c>
+      <c r="F12" t="n">
+        <v>5</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>9</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>2025-Q3</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B13" t="n">
+        <v>4</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" t="n">
+        <v>48</v>
+      </c>
+      <c r="E13" t="n">
+        <v>4</v>
+      </c>
+      <c r="F13" t="n">
+        <v>3</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>3</v>
+      </c>
+      <c r="I13" t="n">
+        <v>7</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>2025-Q4</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" t="n">
+        <v>42</v>
+      </c>
+      <c r="E14" t="n">
+        <v>5</v>
+      </c>
+      <c r="F14" t="n">
+        <v>5</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>4</v>
+      </c>
+      <c r="I14" t="n">
+        <v>4</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>2026-Q1</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B15" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="n">
+        <v>30</v>
+      </c>
+      <c r="E15" t="n">
+        <v>21</v>
+      </c>
+      <c r="F15" t="n">
+        <v>21</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" t="n">
+        <v>9</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>2026-Q2</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B16" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="n">
+        <v>36</v>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="n">
+        <v>2</v>
+      </c>
+      <c r="I16" t="n">
+        <v>5</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>2026-Q3</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B17" t="n">
+        <v>4</v>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>2026-Q4</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -632,7 +1266,7 @@
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>56.64</v>
+        <v>56.58</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -651,7 +1285,7 @@
         <v>2</v>
       </c>
       <c r="D3" t="n">
-        <v>57.17</v>
+        <v>57.11</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -670,7 +1304,7 @@
         <v>3</v>
       </c>
       <c r="D4" t="n">
-        <v>67.52</v>
+        <v>67.45999999999999</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -689,7 +1323,7 @@
         <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>55.23</v>
+        <v>55.17</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -708,7 +1342,7 @@
         <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>66.12</v>
+        <v>66.06999999999999</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -727,7 +1361,7 @@
         <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>70.06999999999999</v>
+        <v>70.02</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -746,7 +1380,7 @@
         <v>3</v>
       </c>
       <c r="D8" t="n">
-        <v>77.67</v>
+        <v>77.62</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -765,7 +1399,7 @@
         <v>4</v>
       </c>
       <c r="D9" t="n">
-        <v>82.51000000000001</v>
+        <v>82.45999999999999</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -860,7 +1494,7 @@
         <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>80.45</v>
+        <v>80.15000000000001</v>
       </c>
       <c r="E14" t="b">
         <v>1</v>
@@ -2193,31 +2827,31 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>385</v>
+        <v>350</v>
       </c>
       <c r="D2" t="n">
-        <v>3715</v>
+        <v>3695</v>
       </c>
       <c r="E2" t="n">
-        <v>613942412587</v>
+        <v>613430343687</v>
       </c>
       <c r="F2" t="n">
-        <v>189</v>
+        <v>180</v>
       </c>
       <c r="G2" t="n">
         <v>27.14</v>
       </c>
       <c r="H2" t="n">
-        <v>78.09</v>
+        <v>76.75</v>
       </c>
       <c r="I2" t="n">
-        <v>84.43000000000001</v>
+        <v>84.48999999999999</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>54.18</v>
+        <v>53.75</v>
       </c>
     </row>
     <row r="3">
@@ -2230,22 +2864,22 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>435</v>
+        <v>398</v>
       </c>
       <c r="D3" t="n">
-        <v>3777</v>
+        <v>3754</v>
       </c>
       <c r="E3" t="n">
-        <v>676307695918</v>
+        <v>675795627018</v>
       </c>
       <c r="F3" t="n">
-        <v>202</v>
+        <v>193</v>
       </c>
       <c r="G3" t="n">
         <v>27.24</v>
       </c>
       <c r="H3" t="n">
-        <v>88.23999999999999</v>
+        <v>87.28</v>
       </c>
       <c r="I3" t="n">
         <v>85.84</v>
@@ -2254,7 +2888,7 @@
         <v>99.97</v>
       </c>
       <c r="K3" t="n">
-        <v>91.34999999999999</v>
+        <v>91.03</v>
       </c>
     </row>
     <row r="4">
@@ -2267,16 +2901,16 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>493</v>
+        <v>456</v>
       </c>
       <c r="D4" t="n">
-        <v>3826</v>
+        <v>3803</v>
       </c>
       <c r="E4" t="n">
-        <v>676325745918</v>
+        <v>675813677018</v>
       </c>
       <c r="F4" t="n">
-        <v>206</v>
+        <v>197</v>
       </c>
       <c r="G4" t="n">
         <v>27.24</v>
@@ -2300,35 +2934,35 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Real (stock activo consolidado)</t>
+          <t>Parcial (no comparable)</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>493</v>
+        <v>437</v>
       </c>
       <c r="D5" t="n">
-        <v>3826</v>
+        <v>3791</v>
       </c>
       <c r="E5" t="n">
-        <v>676325745918</v>
+        <v>674847167117</v>
       </c>
       <c r="F5" t="n">
-        <v>206</v>
+        <v>192</v>
       </c>
       <c r="G5" t="n">
         <v>27.24</v>
       </c>
       <c r="H5" t="n">
-        <v>100</v>
+        <v>95.83</v>
       </c>
       <c r="I5" t="n">
-        <v>86.95999999999999</v>
+        <v>86.68000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>100</v>
+        <v>98.52</v>
       </c>
       <c r="K5" t="n">
-        <v>95.65000000000001</v>
+        <v>93.68000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -2342,627 +2976,106 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>año</t>
+          <t>periodo</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>trimestre</t>
+          <t>establecimientos_activos</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>homicidios</t>
+          <t>empleabilidad_total</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>hurtos</t>
+          <t>ingresos_operacionales</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>siniestralidad</t>
+          <t>cancelaciones_trim</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>lesionados</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>mortales</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>vif</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>rinas</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>periodo</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>spa</t>
+          <t>renovaciones_trim</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>2023</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-Q1</t>
+        </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>446</v>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>3796</v>
       </c>
       <c r="D2" t="n">
-        <v>57</v>
+        <v>675132683017</v>
       </c>
       <c r="E2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F2" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-Q2</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>439</v>
+      </c>
+      <c r="C3" t="n">
+        <v>3792</v>
+      </c>
+      <c r="D3" t="n">
+        <v>675129683017</v>
+      </c>
+      <c r="E3" t="n">
         <v>7</v>
       </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>3</v>
-      </c>
-      <c r="I2" t="n">
+      <c r="F3" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-Q3</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>437</v>
+      </c>
+      <c r="C4" t="n">
+        <v>3791</v>
+      </c>
+      <c r="D4" t="n">
+        <v>674847167117</v>
+      </c>
+      <c r="E4" t="n">
         <v>2</v>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>2023-Q1</t>
-        </is>
-      </c>
-      <c r="K2" t="n">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2023</v>
-      </c>
-      <c r="B3" t="n">
-        <v>2</v>
-      </c>
-      <c r="C3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" t="n">
-        <v>68</v>
-      </c>
-      <c r="E3" t="n">
-        <v>8</v>
-      </c>
-      <c r="F3" t="n">
-        <v>7</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" t="n">
-        <v>2</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>2023-Q2</t>
-        </is>
-      </c>
-      <c r="K3" t="n">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>2023</v>
-      </c>
-      <c r="B4" t="n">
-        <v>3</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" t="n">
-        <v>64</v>
-      </c>
-      <c r="E4" t="n">
-        <v>5</v>
-      </c>
       <c r="F4" t="n">
-        <v>4</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" t="n">
-        <v>2</v>
-      </c>
-      <c r="I4" t="n">
         <v>6</v>
       </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>2023-Q3</t>
-        </is>
-      </c>
-      <c r="K4" t="n">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>2023</v>
-      </c>
-      <c r="B5" t="n">
-        <v>4</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" t="n">
-        <v>56</v>
-      </c>
-      <c r="E5" t="n">
-        <v>9</v>
-      </c>
-      <c r="F5" t="n">
-        <v>8</v>
-      </c>
-      <c r="G5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H5" t="n">
-        <v>2</v>
-      </c>
-      <c r="I5" t="n">
-        <v>4</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>2023-Q4</t>
-        </is>
-      </c>
-      <c r="K5" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B6" t="n">
-        <v>1</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" t="n">
-        <v>61</v>
-      </c>
-      <c r="E6" t="n">
-        <v>7</v>
-      </c>
-      <c r="F6" t="n">
-        <v>5</v>
-      </c>
-      <c r="G6" t="n">
-        <v>2</v>
-      </c>
-      <c r="H6" t="n">
-        <v>5</v>
-      </c>
-      <c r="I6" t="n">
-        <v>4</v>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>2024-Q1</t>
-        </is>
-      </c>
-      <c r="K6" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B7" t="n">
-        <v>2</v>
-      </c>
-      <c r="C7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" t="n">
-        <v>76</v>
-      </c>
-      <c r="E7" t="n">
-        <v>5</v>
-      </c>
-      <c r="F7" t="n">
-        <v>5</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>2024-Q2</t>
-        </is>
-      </c>
-      <c r="K7" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B8" t="n">
-        <v>3</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" t="n">
-        <v>73</v>
-      </c>
-      <c r="E8" t="n">
-        <v>2</v>
-      </c>
-      <c r="F8" t="n">
-        <v>2</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" t="n">
-        <v>3</v>
-      </c>
-      <c r="I8" t="n">
-        <v>6</v>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>2024-Q3</t>
-        </is>
-      </c>
-      <c r="K8" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B9" t="n">
-        <v>4</v>
-      </c>
-      <c r="C9" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" t="n">
-        <v>64</v>
-      </c>
-      <c r="E9" t="n">
-        <v>3</v>
-      </c>
-      <c r="F9" t="n">
-        <v>3</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" t="n">
-        <v>2</v>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>2024-Q4</t>
-        </is>
-      </c>
-      <c r="K9" t="n">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B10" t="n">
-        <v>1</v>
-      </c>
-      <c r="C10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" t="n">
-        <v>48</v>
-      </c>
-      <c r="E10" t="n">
-        <v>9</v>
-      </c>
-      <c r="F10" t="n">
-        <v>9</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" t="n">
-        <v>1</v>
-      </c>
-      <c r="I10" t="n">
-        <v>3</v>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>2025-Q1</t>
-        </is>
-      </c>
-      <c r="K10" t="n">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B11" t="n">
-        <v>2</v>
-      </c>
-      <c r="C11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" t="n">
-        <v>56</v>
-      </c>
-      <c r="E11" t="n">
-        <v>6</v>
-      </c>
-      <c r="F11" t="n">
-        <v>5</v>
-      </c>
-      <c r="G11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H11" t="n">
-        <v>2</v>
-      </c>
-      <c r="I11" t="n">
-        <v>2</v>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>2025-Q2</t>
-        </is>
-      </c>
-      <c r="K11" t="n">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B12" t="n">
-        <v>3</v>
-      </c>
-      <c r="C12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D12" t="n">
-        <v>57</v>
-      </c>
-      <c r="E12" t="n">
-        <v>5</v>
-      </c>
-      <c r="F12" t="n">
-        <v>5</v>
-      </c>
-      <c r="G12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" t="n">
-        <v>9</v>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>2025-Q3</t>
-        </is>
-      </c>
-      <c r="K12" t="n">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B13" t="n">
-        <v>4</v>
-      </c>
-      <c r="C13" t="n">
-        <v>1</v>
-      </c>
-      <c r="D13" t="n">
-        <v>48</v>
-      </c>
-      <c r="E13" t="n">
-        <v>4</v>
-      </c>
-      <c r="F13" t="n">
-        <v>3</v>
-      </c>
-      <c r="G13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" t="n">
-        <v>3</v>
-      </c>
-      <c r="I13" t="n">
-        <v>7</v>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>2025-Q4</t>
-        </is>
-      </c>
-      <c r="K13" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" t="n">
-        <v>42</v>
-      </c>
-      <c r="E14" t="n">
-        <v>5</v>
-      </c>
-      <c r="F14" t="n">
-        <v>5</v>
-      </c>
-      <c r="G14" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" t="n">
-        <v>4</v>
-      </c>
-      <c r="I14" t="n">
-        <v>4</v>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>2026-Q1</t>
-        </is>
-      </c>
-      <c r="K14" t="n">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B15" t="n">
-        <v>2</v>
-      </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="n">
-        <v>30</v>
-      </c>
-      <c r="E15" t="n">
-        <v>21</v>
-      </c>
-      <c r="F15" t="n">
-        <v>21</v>
-      </c>
-      <c r="G15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" t="n">
-        <v>1</v>
-      </c>
-      <c r="I15" t="n">
-        <v>9</v>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>2026-Q2</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B16" t="n">
-        <v>3</v>
-      </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="n">
-        <v>36</v>
-      </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="n">
-        <v>2</v>
-      </c>
-      <c r="I16" t="n">
-        <v>5</v>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>2026-Q3</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B17" t="n">
-        <v>4</v>
-      </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>2026-Q4</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Roosevelt: mostrar 2026 en todas las graficas segun guia Barrio Obrero (cards ultimo anio=2026, movilidad trimestral hasta cobertura real, ITT trimestral 2026 Q1-Q3); corregir peso DesSocial 9%->19%; pesos y scores intactos
</commit_message>
<xml_diff>
--- a/outputs/itt_roosevelt/ITT_Roosevelt_Consolidado.xlsx
+++ b/outputs/itt_roosevelt/ITT_Roosevelt_Consolidado.xlsx
@@ -1223,7 +1223,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1497,6 +1497,44 @@
         <v>80.15000000000001</v>
       </c>
       <c r="E14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-Q2</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" t="n">
+        <v>74.12</v>
+      </c>
+      <c r="E15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-Q3</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C16" t="n">
+        <v>3</v>
+      </c>
+      <c r="D16" t="n">
+        <v>81.76000000000001</v>
+      </c>
+      <c r="E16" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Roosevelt Educacion: consolidado regenerado desde data/Educacion_2026 (nuevo build_educacion_roosevelt.py, valida linea 2023-2025 sin cambios); tablas y graficas muestran 2026 (matricula 2057, repitencia 138, desercion s/d); score ITT 2026 por carry-forward, ITT intacto
</commit_message>
<xml_diff>
--- a/outputs/itt_roosevelt/ITT_Roosevelt_Consolidado.xlsx
+++ b/outputs/itt_roosevelt/ITT_Roosevelt_Consolidado.xlsx
@@ -2647,7 +2647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2782,6 +2782,29 @@
       </c>
       <c r="I4" t="n">
         <v>79.8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B5" t="n">
+        <v>2057</v>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="n">
+        <v>138</v>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="n">
+        <v>6.71</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="n">
+        <v>66.45</v>
+      </c>
+      <c r="I5" t="n">
+        <v>66.40000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>